<commit_message>
fixed PX4310 contact time
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627_v2.xlsx
+++ b/AssessmentSchedule_2627_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="8_{0C641013-E594-4AA6-B777-C2C249EA34A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2422B9DF-796A-46F0-B2F2-91CCAA23F76D}"/>
+  <xr:revisionPtr revIDLastSave="249" documentId="8_{0C641013-E594-4AA6-B777-C2C249EA34A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FBA324E-4652-42BF-A934-EF70E5B8E75B}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" activeTab="2" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" activeTab="1" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -30175,7 +30175,7 @@
         <v>0.5</v>
       </c>
       <c r="G61" s="31">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="H61" s="31">
         <v>1</v>
@@ -30246,7 +30246,7 @@
       </c>
       <c r="AE61" s="37">
         <f>SUM(Table14[[#This Row],[Autumn Week 1]:[Spring Week 12]])</f>
-        <v>29.5</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="62" spans="1:31">
@@ -37969,15 +37969,15 @@
       </c>
       <c r="D67">
         <f>INDEX(Table14[Total],MATCH(Sheet2!A67,Table14[Module Code],0))</f>
-        <v>29.5</v>
+        <v>12.5</v>
       </c>
       <c r="E67">
         <f t="shared" si="0"/>
-        <v>530.90000000000009</v>
+        <v>513.90000000000009</v>
       </c>
       <c r="F67">
         <f t="shared" si="1"/>
-        <v>8.8483333333333345</v>
+        <v>8.5650000000000013</v>
       </c>
     </row>
     <row r="68" spans="1:6">

</xml_diff>